<commit_message>
corrections to inverse values added timestamp to excel extract name
</commit_message>
<xml_diff>
--- a/Kwartaalrapportage/Aggregation_Results.xlsx
+++ b/Kwartaalrapportage/Aggregation_Results.xlsx
@@ -463,16 +463,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>253076.67</v>
+        <v>-253076.67</v>
       </c>
       <c r="C2" t="n">
-        <v>-242183.81</v>
+        <v>242183.81</v>
       </c>
       <c r="D2" t="n">
-        <v>333655.29</v>
+        <v>-333655.29</v>
       </c>
       <c r="E2" t="n">
-        <v>329713.07</v>
+        <v>-329713.07</v>
       </c>
     </row>
     <row r="3">
@@ -501,16 +501,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-1815040.82</v>
+        <v>856550.58</v>
       </c>
       <c r="C4" t="n">
-        <v>-252414.59</v>
+        <v>252414.59</v>
       </c>
       <c r="D4" t="n">
-        <v>-66944.20999999999</v>
+        <v>66944.20999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>-4478.240000000002</v>
+        <v>4478.240000000002</v>
       </c>
     </row>
     <row r="5">
@@ -520,16 +520,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-72229.00999999999</v>
+        <v>72229.00999999999</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>-1704805.9</v>
+        <v>1704805.9</v>
       </c>
       <c r="E5" t="n">
-        <v>-46195.68</v>
+        <v>46195.68</v>
       </c>
     </row>
     <row r="6">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-130732.05</v>
+        <v>130732.05</v>
       </c>
       <c r="C7" t="n">
-        <v>-159293.52</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>-9832.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>298</v>
+        <v>-298</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>-12</v>
+        <v>12</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>118011.22</v>
+        <v>-118011.22</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>215656.07</v>
+        <v>-215656.07</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1185,7 +1185,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>-50000</v>
+        <v>50000</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>-150000</v>
+        <v>150000</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>-1504805.9</v>
+        <v>1504805.9</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>565.61</v>
+        <v>-565.61</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1309,7 +1309,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2819.5</v>
+        <v>-2819.5</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>341.17</v>
+        <v>-341.17</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2570.42</v>
+        <v>-2570.42</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>-93671.36</v>
+        <v>93671.36</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>21311</v>
+        <v>-21311</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3598.75</v>
+        <v>-3598.75</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>-4777.299999999988</v>
+        <v>4777.299999999988</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -2270,7 +2270,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>-100</v>
+        <v>100</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>175043.7</v>
+        <v>-175043.7</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>78132.97</v>
+        <v>-78132.97</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2363,7 +2363,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>-16000</v>
+        <v>16000</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2394,7 +2394,7 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>-55056.9</v>
+        <v>55056.9</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>-1172.11</v>
+        <v>1172.11</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2456,7 +2456,7 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>6106.17</v>
+        <v>-6106.17</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>-623388.77</v>
+        <v>623388.77</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2518,7 +2518,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>6075.83</v>
+        <v>-6075.83</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2549,7 +2549,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>-4325.55</v>
+        <v>4325.55</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>633.75</v>
+        <v>-633.75</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2704,7 +2704,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>-11223.9</v>
+        <v>11223.9</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2735,7 +2735,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>-1090432.03</v>
+        <v>131941.79</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2766,7 +2766,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>-115142.32</v>
+        <v>115142.32</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2797,7 +2797,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>-6451.380000000001</v>
+        <v>6451.380000000001</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2828,7 +2828,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>390</v>
+        <v>-390</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2859,7 +2859,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>3371</v>
+        <v>-3371</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2890,7 +2890,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>16279.01</v>
+        <v>-16279.01</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2921,7 +2921,7 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>-33.39</v>
+        <v>33.39</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2952,7 +2952,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>-100940.4</v>
+        <v>100940.4</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>120508.93</v>
+        <v>-120508.93</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -3014,7 +3014,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>-16469.5</v>
+        <v>16469.5</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>1.73</v>
+        <v>-1.73</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -3076,7 +3076,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>6251.360000000001</v>
+        <v>-6251.360000000001</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -3107,7 +3107,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>-3040.89</v>
+        <v>3040.89</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -3138,7 +3138,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>-10229.54</v>
+        <v>10229.54</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -3169,7 +3169,7 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>-959.22</v>
+        <v>959.22</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -3200,7 +3200,7 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>-117821.23</v>
+        <v>117821.23</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -3231,7 +3231,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>-1741.9</v>
+        <v>1741.9</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>-1500</v>
+        <v>1500</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3293,7 +3293,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>-720</v>
+        <v>720</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>-300</v>
+        <v>300</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -3355,7 +3355,7 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>-670.63</v>
+        <v>670.63</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -3386,7 +3386,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -4285,7 +4285,7 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>-500</v>
+        <v>500</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -4316,7 +4316,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>-12</v>
+        <v>12</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>126011.32</v>
+        <v>-126011.32</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
@@ -4378,7 +4378,7 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>203713.75</v>
+        <v>-203713.75</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -4409,7 +4409,7 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>-46195.68</v>
+        <v>46195.68</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -4440,7 +4440,7 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>500</v>
+        <v>-500</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -4471,7 +4471,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>-250</v>
+        <v>250</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -4595,7 +4595,7 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>-19084.01</v>
+        <v>19084.01</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
@@ -4626,7 +4626,7 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>16329.55</v>
+        <v>-16329.55</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -4657,7 +4657,7 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>-1032.18</v>
+        <v>1032.18</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
@@ -4688,7 +4688,7 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>1582.08</v>
+        <v>-1582.08</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -4719,7 +4719,7 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -4750,7 +4750,7 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>-43084.22</v>
+        <v>43084.22</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -4781,7 +4781,7 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>47925.38</v>
+        <v>-47925.38</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>-428.4</v>
+        <v>428.4</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -4843,7 +4843,7 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>-6436.44</v>
+        <v>6436.44</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -4874,7 +4874,7 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>-9832.52</v>
+        <v>0</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="F159" t="n">
-        <v>-413462</v>
+        <v>413462</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -5618,7 +5618,7 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>149</v>
+        <v>-149</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -5649,7 +5649,7 @@
         </is>
       </c>
       <c r="F161" t="n">
-        <v>-12</v>
+        <v>12</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -5680,7 +5680,7 @@
         </is>
       </c>
       <c r="F162" t="n">
-        <v>116640.65</v>
+        <v>-116640.65</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
@@ -5711,7 +5711,7 @@
         </is>
       </c>
       <c r="F163" t="n">
-        <v>54649.54</v>
+        <v>-54649.54</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
@@ -5742,7 +5742,7 @@
         </is>
       </c>
       <c r="F164" t="n">
-        <v>4455.51</v>
+        <v>-4455.51</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
         </is>
       </c>
       <c r="F165" t="n">
-        <v>-900</v>
+        <v>900</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -5897,7 +5897,7 @@
         </is>
       </c>
       <c r="F169" t="n">
-        <v>-240030.54</v>
+        <v>240030.54</v>
       </c>
       <c r="G169" t="inlineStr">
         <is>
@@ -5928,7 +5928,7 @@
         </is>
       </c>
       <c r="F170" t="n">
-        <v>1792</v>
+        <v>-1792</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -5959,7 +5959,7 @@
         </is>
       </c>
       <c r="F171" t="n">
-        <v>16721.33</v>
+        <v>-16721.33</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
@@ -5990,7 +5990,7 @@
         </is>
       </c>
       <c r="F172" t="n">
-        <v>-94827.03999999999</v>
+        <v>94827.03999999999</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
@@ -6021,7 +6021,7 @@
         </is>
       </c>
       <c r="F173" t="n">
-        <v>76731.09</v>
+        <v>-76731.09</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
@@ -6052,7 +6052,7 @@
         </is>
       </c>
       <c r="F174" t="n">
-        <v>-16505.94</v>
+        <v>16505.94</v>
       </c>
       <c r="G174" t="inlineStr">
         <is>
@@ -6083,7 +6083,7 @@
         </is>
       </c>
       <c r="F175" t="n">
-        <v>-159293.52</v>
+        <v>0</v>
       </c>
       <c r="G175" t="inlineStr">
         <is>

</xml_diff>